<commit_message>
Update lab schedule to separate P2-2 and P2-3 into distinct weeks; adjust lab rows in schedule generation script
</commit_message>
<xml_diff>
--- a/Weekly Schedules.xlsx
+++ b/Weekly Schedules.xlsx
@@ -690,7 +690,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>P2-2/P2-3</t>
+          <t>P2-2</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
@@ -711,14 +711,10 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Lab 7 (Lecture 26 or later)</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Lab 7: Lab6 in-lab activity submission</t>
-        </is>
-      </c>
+          <t>P2-3</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -734,8 +730,16 @@
           <t>Lecture 30: Issues with Hypothesis Testing 2: Multiple comparisons; Lecture 31: Beyond Recipes: Frequentist and Bayesian Approaches to Statistical Modeling; Lecture 32: Frequentist modeling using the likelihood function</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Lab 7 (Lecture 26 or later)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Lab 7: Lab6 in-lab activity submission</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">

</xml_diff>

<commit_message>
Update lab summary and weekly schedule to reflect changes in lab topics and lecture alignment
</commit_message>
<xml_diff>
--- a/Weekly Schedules.xlsx
+++ b/Weekly Schedules.xlsx
@@ -430,7 +430,7 @@
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="37" customWidth="1" min="2" max="2"/>
     <col width="80" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
     <col width="73" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -573,7 +573,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Lab 4 (Lecture 9 or 10)</t>
+          <t>Lab 4 (Lecture 11)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -598,7 +598,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Lab 5 (Lecture 15 or 16)</t>
+          <t>Lab 5 (Lecture 14)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -665,7 +665,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Lab 6 (Lecture 18 or 20)</t>
+          <t>Lab 6 (Lecture 22)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -732,7 +732,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Lab 7 (Lecture 26 or later)</t>
+          <t>Lab 7 (Lecture 30)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">

</xml_diff>

<commit_message>
Update lab deliverables and project schedule
</commit_message>
<xml_diff>
--- a/Weekly Schedules.xlsx
+++ b/Weekly Schedules.xlsx
@@ -431,7 +431,7 @@
     <col width="37" customWidth="1" min="2" max="2"/>
     <col width="80" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="73" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -480,11 +480,7 @@
           <t>Lab 1 (Lecture 1)</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Lab 1: Lab1 in-lab activity submission | Tutorial 1 (pre-lab for lab2)</t>
-        </is>
-      </c>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -507,7 +503,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Lab 2: Lab2 in-lab activity submission | Tutorial 2 (pre-lab for lab3)</t>
+          <t>Lab 2: Lab1 in-lab activity submission | Tutorial 1 | Tutorial 2 (pre-lab for lab2)</t>
         </is>
       </c>
     </row>
@@ -532,7 +528,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Lab 3: Lab3 in-lab activity submission | Tutorial 3 (pre-lab for lab4)</t>
+          <t>Lab 3: Lab2 in-lab activity submission | Tutorial 3 (pre-lab for lab3)</t>
         </is>
       </c>
     </row>
@@ -555,7 +551,11 @@
           <t>P1-1 (Lecture 8)</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>P1-1: Lab3 in-lab activity submission</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -578,7 +578,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Lab 4: Lab4 in-lab activity submission | Tutorial 4 (pre-lab for lab5)</t>
+          <t>Lab 4: Project 1 Outline | Tutorial 4 (pre-lab for lab4)</t>
         </is>
       </c>
     </row>
@@ -603,7 +603,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Lab 5: Lab5 in-lab activity submission | Tutorial 5 (pre-lab for lab6)</t>
+          <t>Lab 5: Lab4 in-lab activity submission | Tutorial 5 (pre-lab for lab5)</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,11 @@
           <t>P1-2</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>P1-2: Lab5 in-lab activity submission</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -647,7 +651,11 @@
           <t>P2-1</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>P2-1: P1 Video</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -670,7 +678,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Lab 6: Lab6 in-lab activity submission | Tutorial 6 (pre-lab for lab7)</t>
+          <t>Lab 6: Lab6 in-lab activity submission | Tutorial 6 (pre-lab for lab6) | P2 Outline</t>
         </is>
       </c>
     </row>
@@ -693,7 +701,11 @@
           <t>P2-2</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>P2-2: Lab6 in-lab activity submission</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -714,7 +726,11 @@
           <t>P2-3</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>P2-3: P2 Progress Report</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -737,7 +753,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Lab 7: Lab7 in-lab activity submission</t>
+          <t>Lab 7: P2 writeup | Tutorial 7 (pre-lab for lab7)</t>
         </is>
       </c>
     </row>
@@ -755,8 +771,16 @@
           <t>Quiz 4; Lecture 33: Bayesian modeling with discrete distributions; Lecture 34: Bayesian modeling with the beta-binomial model</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Lab 8</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Lab 8: P2 Resubmission</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">

</xml_diff>